<commit_message>
corrections pour validté  schematron & PDF/A3
</commit_message>
<xml_diff>
--- a/clients.xlsx
+++ b/clients.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\__dev_projects\ez_facture_excel\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\__dev_projects\ezfacture\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D539813C-A213-4F57-9C02-5A2218505D22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{561C8AC8-2E2F-444C-A9B9-77A1A435F92E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{3720E7CA-D5CC-410F-BB8F-0B593B646E11}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="43">
   <si>
     <t>C00001</t>
   </si>
@@ -47,9 +47,6 @@
     <t>SARL Dubois</t>
   </si>
   <si>
-    <t xml:space="preserve"> </t>
-  </si>
-  <si>
     <t>Durand</t>
   </si>
   <si>
@@ -165,6 +162,9 @@
   </si>
   <si>
     <t>Remarques</t>
+  </si>
+  <si>
+    <t>FR12123456789</t>
   </si>
 </sst>
 </file>
@@ -268,7 +268,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -315,6 +315,14 @@
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
@@ -742,18 +750,17 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="dotted">
-          <color auto="1"/>
-        </left>
-        <right style="dotted">
-          <color auto="1"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="dotted">
+          <color auto="1"/>
+        </left>
+        <right style="dotted">
+          <color auto="1"/>
+        </right>
+        <top/>
+        <bottom/>
       </border>
       <protection locked="0" hidden="0"/>
     </dxf>
@@ -1293,7 +1300,7 @@
     <col min="2" max="2" width="13.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="6.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.85546875" style="16" customWidth="1"/>
     <col min="6" max="6" width="19.5703125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="8.140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="10.5703125" bestFit="1" customWidth="1"/>
@@ -1313,70 +1320,70 @@
   <sheetData>
     <row r="1" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="J1" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="K1" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="L1" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="N1" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="O1" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="P1" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="P1" s="4" t="s">
+      <c r="Q1" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="R1" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="S1" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="S1" s="5" t="s">
+      <c r="T1" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="T1" s="3" t="s">
+      <c r="U1" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="U1" s="3" t="s">
+      <c r="V1" s="6" t="s">
         <v>41</v>
-      </c>
-      <c r="V1" s="6" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.25">
@@ -1389,113 +1396,113 @@
       <c r="C2" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="D2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E2" s="15">
+        <v>12345678900012</v>
+      </c>
+      <c r="F2" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="G2" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="F2" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="G2" s="9" t="s">
+      <c r="H2" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="9" t="s">
+      <c r="I2" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="I2" s="8" t="s">
+      <c r="J2" s="8" t="s">
         <v>6</v>
-      </c>
-      <c r="J2" s="8" t="s">
-        <v>7</v>
       </c>
       <c r="K2" s="10">
         <v>44000</v>
       </c>
       <c r="L2" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="M2" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="M2" s="8" t="s">
+      <c r="N2" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="N2" s="8" t="s">
+      <c r="O2" s="8" t="s">
         <v>10</v>
-      </c>
-      <c r="O2" s="8" t="s">
-        <v>11</v>
       </c>
       <c r="P2" s="10">
         <v>44000</v>
       </c>
       <c r="Q2" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="R2" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="R2" s="8" t="s">
-        <v>9</v>
-      </c>
       <c r="S2" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="T2" s="12" t="s">
         <v>12</v>
-      </c>
-      <c r="T2" s="12" t="s">
-        <v>13</v>
       </c>
       <c r="U2" s="8"/>
       <c r="V2" s="13"/>
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="C3" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="D3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E3" s="15">
+        <v>12345678900012</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="G3" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="E3" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="F3" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="G3" s="9" t="s">
+      <c r="H3" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="H3" s="9" t="s">
+      <c r="I3" s="8" t="s">
         <v>18</v>
-      </c>
-      <c r="I3" s="8" t="s">
-        <v>19</v>
       </c>
       <c r="J3" s="8"/>
       <c r="K3" s="10">
         <v>75001</v>
       </c>
       <c r="L3" s="8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="M3" s="8" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="N3" s="8" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="O3" s="8"/>
       <c r="P3" s="10">
         <v>75001</v>
       </c>
       <c r="Q3" s="8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="R3" s="8" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="S3" s="11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="T3" s="8"/>
       <c r="U3" s="8"/>

</xml_diff>